<commit_message>
Subir archivos actuales del proyecto erp-ins-kpis
</commit_message>
<xml_diff>
--- a/reporte_siges_salud.xlsx
+++ b/reporte_siges_salud.xlsx
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7.5</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>38.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>169.5</v>
+        <v>116.25</v>
       </c>
     </row>
     <row r="8">
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>16</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -642,10 +642,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>202602</v>
+        <v>202604</v>
       </c>
       <c r="D2" t="n">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -665,14 +665,14 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>202602</v>
+        <v>202604</v>
       </c>
       <c r="D3" t="n">
-        <v>70.75</v>
+        <v>119</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PROC.RM</t>
+          <t>PROC.BI</t>
         </is>
       </c>
     </row>
@@ -688,14 +688,14 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>202602</v>
+        <v>202604</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>27.25</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PROC.SWAT</t>
+          <t>PROC.RM</t>
         </is>
       </c>
     </row>
@@ -707,14 +707,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>095-400-INS-REG</t>
+          <t>095-202-RDIG</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>202602</v>
+        <v>202604</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -725,19 +725,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PROC.SWAT</t>
+          <t>PROC.SALUD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>151-350-NV.OP.SWAT</t>
+          <t>095-400-INS-REG</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>202602</v>
+        <v>202604</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5</v>
+        <v>8</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -748,23 +748,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PROC.SALUD</t>
+          <t>PROC.SWAT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>151-400-RGT2.0</t>
+          <t>151-350-NV.OP.SWAT</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>202602</v>
+        <v>202604</v>
       </c>
       <c r="D7" t="n">
-        <v>38.5</v>
+        <v>16</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PROC.QA</t>
+          <t>PROC.SWAT</t>
         </is>
       </c>
     </row>
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>202602</v>
+        <v>202604</v>
       </c>
       <c r="D8" t="n">
-        <v>55.75</v>
+        <v>6</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PROC.RM</t>
+          <t>PROC.QA</t>
         </is>
       </c>
     </row>
@@ -799,18 +799,18 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>579-203-REDIMED</t>
+          <t>151-400-RGT2.0</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>202602</v>
+        <v>202604</v>
       </c>
       <c r="D9" t="n">
-        <v>16</v>
+        <v>60.5</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>PROC.BI</t>
+          <t>PROC.RM</t>
         </is>
       </c>
     </row>
@@ -826,12 +826,35 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>202602</v>
+        <v>202604</v>
       </c>
       <c r="D10" t="n">
-        <v>41.5</v>
+        <v>17</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>PROC.BI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PROC.SALUD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>579-203-REDIMED</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>202604</v>
+      </c>
+      <c r="D11" t="n">
+        <v>27.75</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>PROC.RM</t>
         </is>

</xml_diff>